<commit_message>
Make CSV formatted tables
Add descriptions to accession table; create tables for manuscript as CSVs
</commit_message>
<xml_diff>
--- a/Results/Tables/Table S1 leaf_surface_supp_table_accession_list.xlsx
+++ b/Results/Tables/Table S1 leaf_surface_supp_table_accession_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madisonplunkert/Documents/Lowry Lab/Salt Spray/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madisonplunkert/Documents/GitHub/Salt-spray-adaptation-2025/Results/Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FA40E5-21CA-2847-AE2A-BDF789266BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09391D88-617D-8C41-9695-444B46CD0154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="920" windowWidth="27640" windowHeight="16400" xr2:uid="{3CC583D9-CC0E-C947-8CC1-66B8A88126C1}"/>
+    <workbookView xWindow="5940" yWindow="740" windowWidth="27640" windowHeight="16400" xr2:uid="{3CC583D9-CC0E-C947-8CC1-66B8A88126C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Accession_list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>Population_Code</t>
   </si>
@@ -102,6 +102,39 @@
   </si>
   <si>
     <t>inland</t>
+  </si>
+  <si>
+    <t>Population_Name</t>
+  </si>
+  <si>
+    <t>Bodega Headlands</t>
+  </si>
+  <si>
+    <t>Pacific Grove</t>
+  </si>
+  <si>
+    <t>Sperm Whale Beach</t>
+  </si>
+  <si>
+    <t>Toro County Park</t>
+  </si>
+  <si>
+    <t>Sweet Creek Road</t>
+  </si>
+  <si>
+    <t>Rogue River</t>
+  </si>
+  <si>
+    <t>Heceta Beach</t>
+  </si>
+  <si>
+    <t>Lower Mendocino County</t>
+  </si>
+  <si>
+    <t>Occidental Arts and Ecology Center</t>
+  </si>
+  <si>
+    <t>Otter Point State Park beach</t>
   </si>
 </sst>
 </file>
@@ -473,229 +506,263 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D496A856-798D-D240-BA9D-DBA79E61827B}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>19</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>38.307032999999997</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>-123.05841700000001</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>4</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>44.135066999999999</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>-124.1228</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4">
         <v>24</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>38.863982999999998</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>-123.083917</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5">
         <v>19</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>38.411267000000002</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>-122.959717</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>3</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>42.464016999999998</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>-124.422917</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>3</v>
+      <c r="B7" t="s">
+        <v>24</v>
       </c>
       <c r="C7">
         <v>3</v>
       </c>
       <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
         <v>36.627991666699998</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>-121.92083</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
         <v>27</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>42.489249999999998</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>-124.2084</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9">
         <v>4</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>2</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>39.035983000000002</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>-123.690467</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
         <v>16</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>7</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>43.959466999999997</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>-123.90245</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="B11">
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
         <v>3</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>2</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>36.603042000000002</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>-121.688408</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>